<commit_message>
docs: atualizado planilha, plano e issues de ExampleGenerator
</commit_message>
<xml_diff>
--- a/entrega1/hygor/planilha-oraculos-matriz-ExampleGenerator.xlsx
+++ b/entrega1/hygor/planilha-oraculos-matriz-ExampleGenerator.xlsx
@@ -464,6 +464,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -478,7 +479,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTA('Matriz de casos'!A5:A52)</f>
+        <f>COUNTA('Matriz de casos'!A5:A58)</f>
         <v/>
       </c>
     </row>
@@ -489,7 +490,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Matriz de casos'!H5:H52,"PASS")+COUNTIF('Matriz de casos'!H5:H52,"FAIL")</f>
+        <f>COUNTIF('Matriz de casos'!H5:H58,"PASS")+COUNTIF('Matriz de casos'!H5:H58,"FAIL")</f>
         <v/>
       </c>
     </row>
@@ -500,7 +501,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Matriz de casos'!H5:H52,"PASS")</f>
+        <f>COUNTIF('Matriz de casos'!H5:H58,"PASS")</f>
         <v/>
       </c>
     </row>
@@ -511,7 +512,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>COUNTIF('Matriz de casos'!H5:H52,"FAIL")</f>
+        <f>COUNTIF('Matriz de casos'!H5:H58,"FAIL")</f>
         <v/>
       </c>
     </row>
@@ -522,7 +523,7 @@
         </is>
       </c>
       <c r="B8">
-        <f>SUM('Matriz de casos'!L5:L52)</f>
+        <f>SUM('Matriz de casos'!L5:L58)</f>
         <v/>
       </c>
     </row>
@@ -534,7 +535,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>6 (CT-EG-24 x2, CT-EG-25, CT-EG-29, CT-EG-45, CT-EG-48)</t>
+          <t>7 (CT-EG-24 x2, CT-EG-25, CT-EG-29, CT-EG-45, CT-EG-48, CT-EG-52)</t>
         </is>
       </c>
     </row>
@@ -550,6 +551,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
@@ -607,6 +609,7 @@
         <v>11</v>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
@@ -622,7 +625,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>97% (1136/1173)</t>
+          <t>97% (1140/1173)</t>
         </is>
       </c>
     </row>
@@ -634,7 +637,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>84% (167/198)</t>
+          <t>90% (179/198)</t>
         </is>
       </c>
     </row>
@@ -646,7 +649,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>96% (255/266)</t>
+          <t>97% (257/266)</t>
         </is>
       </c>
     </row>
@@ -662,6 +665,7 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
@@ -1161,7 +1165,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L52"/>
+  <dimension ref="A1:L58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1188,7 +1192,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Executada em 12/10/2026 via Maven (Surefire), commit ef964b04480889ef86b56cfae84ade8ad4c91c41. Casos parametrizados contam como um caso normativo; a coluna L mostra quantas invocações o JUnit executou. Coluna J: família de defeito (ver aba Defeitos).</t>
+          <t>Executada em 12/10/2026 via Maven (Surefire), commit ef964b04480889ef86b56cfae84ade8ad4c91c41. Casos parametrizados contam como um caso normativo; a coluna L mostra quantas invocações o JUnit executou. Coluna J: família de defeito (ver aba Defeitos). Os casos CT-EG-49 a CT-EG-54 foram projetados depois da primeira medição de cobertura, para os ramos ainda não exercitados; cada um tem justificativa funcional (regra da coluna C).</t>
         </is>
       </c>
     </row>
@@ -2112,22 +2116,22 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Partição: string sem default, enum ou formato</t>
+          <t>Partição: string sem default/enum, formato ausente ou não tratado (parametrizado)</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>propriedade nickname: string</t>
+          <t>propriedade nickname: string com format ausente, email, password</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>"nickname"</t>
+          <t>"nickname" nos 3 casos</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>Conforme esperado</t>
+          <t>Conforme esperado (3/3)</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -2147,7 +2151,7 @@
         </is>
       </c>
       <c r="L20" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21">
@@ -3300,22 +3304,22 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Partição: oneOf com ref inválido primeiro</t>
+          <t>Partição: oneOf/anyOf com ref inválido primeiro (parametrizado)</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>oneOf [Missing, Cat, Dog]</t>
+          <t>oneOf [Missing, Cat, Dog]; anyOf [Missing, Cat, Dog]</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>kind = cat</t>
+          <t>kind = cat nos dois casos</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>Conforme esperado</t>
+          <t>Conforme esperado (2/2)</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
@@ -3326,7 +3330,7 @@
       <c r="I41" s="3" t="inlineStr"/>
       <c r="J41" s="3" t="inlineStr">
         <is>
-          <t>oneOfUsesFirstResolvableAlternative</t>
+          <t>firstResolvableAlternative</t>
         </is>
       </c>
       <c r="K41" s="3" t="inlineStr">
@@ -3335,7 +3339,7 @@
         </is>
       </c>
       <c r="L41" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42">
@@ -3692,22 +3696,22 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Partição: example primitivo só em XML</t>
+          <t>Partição: example primitivo por tipo de mídia (parametrizado)</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>example "pong", {xml}</t>
+          <t>example "pong" com produces {xml}; {text/plain}; {*/*}</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>[{output: none}]</t>
+          <t>output none; output none; "pong" como JSON</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>Conforme esperado</t>
+          <t>Conforme esperado (3/3)</t>
         </is>
       </c>
       <c r="H48" s="4" t="inlineStr">
@@ -3718,7 +3722,7 @@
       <c r="I48" s="3" t="inlineStr"/>
       <c r="J48" s="3" t="inlineStr">
         <is>
-          <t>primitiveExampleAsXmlOnly</t>
+          <t>primitiveExampleByMediaType</t>
         </is>
       </c>
       <c r="K48" s="3" t="inlineStr">
@@ -3727,7 +3731,7 @@
         </is>
       </c>
       <c r="L48" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="49">
@@ -3959,6 +3963,346 @@
         </is>
       </c>
       <c r="L52" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>CT-EG-49</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Saída e mídia</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>R05</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>Valor-limite: schema nulo (parametrizado)</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>generate(null, [json]|[xml], (Schema) null)</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>[{output: none}]</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>Conforme esperado (2/2)</t>
+        </is>
+      </c>
+      <c r="H53" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I53" s="3" t="inlineStr"/>
+      <c r="J53" s="3" t="inlineStr">
+        <is>
+          <t>nullProperty</t>
+        </is>
+      </c>
+      <c r="K53" s="3" t="inlineStr">
+        <is>
+          <t>OutputStructure</t>
+        </is>
+      </c>
+      <c r="L53" s="3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>CT-EG-50</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Precedência</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>R08</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>Valor-limite: enum vazio</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>enum [] sem default</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>"nickname" (nome da propriedade)</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>Conforme esperado</t>
+        </is>
+      </c>
+      <c r="H54" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I54" s="3" t="inlineStr"/>
+      <c r="J54" s="3" t="inlineStr">
+        <is>
+          <t>emptyEnumFallsBackToName</t>
+        </is>
+      </c>
+      <c r="K54" s="3" t="inlineStr">
+        <is>
+          <t>ValuePrecedence</t>
+        </is>
+      </c>
+      <c r="L54" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>CT-EG-51</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>Modelos</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>R12</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>Partição: schema sem tipo (any type)</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>Box{content: {}, id example 4}</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>Geração continua; content presente; id = 4</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>Conforme esperado</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I55" s="3" t="inlineStr"/>
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>anyTypeProperty</t>
+        </is>
+      </c>
+      <c r="K55" s="3" t="inlineStr">
+        <is>
+          <t>Models</t>
+        </is>
+      </c>
+      <c r="L55" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>CT-EG-52</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Modelos</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>R12</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>Partição: modelo de nível superior object sem propriedades</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>Anything: type object</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>Objeto JSON</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>null (resolveModelToExample devolve null)</t>
+        </is>
+      </c>
+      <c r="H56" s="5" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I56" s="3" t="inlineStr">
+        <is>
+          <t>F4</t>
+        </is>
+      </c>
+      <c r="J56" s="3" t="inlineStr">
+        <is>
+          <t>emptyTopLevelObjectModel</t>
+        </is>
+      </c>
+      <c r="K56" s="3" t="inlineStr">
+        <is>
+          <t>Models</t>
+        </is>
+      </c>
+      <c r="L56" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>CT-EG-53</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Composição</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>R13</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>Estrutura: allOf aninhado (allOf de allOf)</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>Outer allOf [allOf[{a},{b}], {c}]</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>a = 1, b = 2, c = 3</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>Conforme esperado</t>
+        </is>
+      </c>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I57" s="3" t="inlineStr"/>
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>nestedAllOf</t>
+        </is>
+      </c>
+      <c r="K57" s="3" t="inlineStr">
+        <is>
+          <t>Models</t>
+        </is>
+      </c>
+      <c r="L57" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>CT-EG-54</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>Composição</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>R12</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>Partição: allOf com $ref inexistente</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>Dog allOf [Missing, {barks}]</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>Sem exceção; barks = true</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>Conforme esperado</t>
+        </is>
+      </c>
+      <c r="H58" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I58" s="3" t="inlineStr"/>
+      <c r="J58" s="3" t="inlineStr">
+        <is>
+          <t>allOfWithDanglingReference</t>
+        </is>
+      </c>
+      <c r="K58" s="3" t="inlineStr">
+        <is>
+          <t>Models</t>
+        </is>
+      </c>
+      <c r="L58" s="3" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4169,22 +4513,22 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>CT-EG-48</t>
+          <t>CT-EG-48, CT-EG-52</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Propriedade type: object sem properties (e $ref inexistente) gera a string "{}" em vez de um objeto JSON.</t>
+          <t>type: object sem properties gera exemplo com tipo errado: a string "{}" quando é propriedade (CT-EG-48; o mesmo vale para $ref inexistente) e null quando é modelo de nível superior (CT-EG-52).</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>resolvePropertyToExample devolve o literal String "{}", que o Json.pretty serializa como string.</t>
+          <t>resolvePropertyToExample devolve o literal String "{}", que o Json.pretty serializa como string; resolveModelToExample devolve null para modelo sem properties, sem composição e que não é array/enum.</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Sim, passo 6 (metadata: "{}").</t>
+          <t>Propriedade: sim, passo 6 (metadata: "{}"). Modelo de nível superior: não; pela CLI o modelo é "desembrulhado" (unaliasSchema) e a operação fica sem Example data.</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -4214,7 +4558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4254,7 +4598,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>resolveModelToExample grava o exemplo gerado no schema de entrada (schema.setExample(values)): o modelo OpenAPI é alterado como efeito colateral, e chamadas seguintes devolvem o exemplo gravado (é o que faz CT-EG-40 passar).</t>
+          <t>resolveModelToExample grava o exemplo gerado no schema de entrada (schema.setExample(values)): o modelo OpenAPI é alterado como efeito colateral, e chamadas seguintes devolvem o exemplo gravado (é o que faz CT-EG-40 passar). Confirmado por execução: example do schema passa de null para {id=1} após generate.</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -4288,7 +4632,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>oneOf/anyOf sem nenhuma alternativa resolvível gera o exemplo "null".</t>
+          <t>oneOf/anyOf sem nenhuma alternativa resolvível gera o exemplo "null" (confirmado por execução em 12/10/2026).</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -4328,6 +4672,23 @@
       <c r="C8" s="3" t="inlineStr">
         <is>
           <t>Mesmo oráculo de R07, mas deixado para a Entrega 2 para manter o escopo da Entrega 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>E6</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>generate(null, mediaTypes, (String) null) — nome de modelo nulo — devolve "Custom MIME type example not yet supported: application/json", mensagem que diz que JSON não é suportado.</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Nenhuma fonte define a saída para modelo nulo; o caso foi projetado para CT-EG-49 e retirado da suíte normativa por falta de oráculo.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: adicionado links das issues de ExampleGenerator
</commit_message>
<xml_diff>
--- a/entrega1/hygor/planilha-oraculos-matriz-ExampleGenerator.xlsx
+++ b/entrega1/hygor/planilha-oraculos-matriz-ExampleGenerator.xlsx
@@ -464,7 +464,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -551,7 +550,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
@@ -609,7 +607,6 @@
         <v>11</v>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
@@ -665,7 +662,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
@@ -1192,7 +1188,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Executada em 12/10/2026 via Maven (Surefire), commit ef964b04480889ef86b56cfae84ade8ad4c91c41. Casos parametrizados contam como um caso normativo; a coluna L mostra quantas invocações o JUnit executou. Coluna J: família de defeito (ver aba Defeitos). Os casos CT-EG-49 a CT-EG-54 foram projetados depois da primeira medição de cobertura, para os ramos ainda não exercitados; cada um tem justificativa funcional (regra da coluna C).</t>
+          <t>Executada em 12/10/2026 via Maven (Surefire), commit ef964b04480889ef86b56cfae84ade8ad4c91c41. Casos parametrizados contam como um caso normativo; a coluna L mostra quantas invocações o JUnit executou. Coluna I: família de defeito (ver aba Defeitos: F1 #25234, F2 #25235, F3 #25236, F4 #25237, repositório oficial). Os casos CT-EG-49 a CT-EG-54 foram projetados depois da primeira medição de cobertura, para os ramos ainda não exercitados; cada um tem justificativa funcional (regra da coluna C).</t>
         </is>
       </c>
     </row>
@@ -4417,7 +4413,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>[preencher nº]</t>
+          <t>#25234</t>
         </is>
       </c>
     </row>
@@ -4459,7 +4455,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>[preencher nº]</t>
+          <t>#25235</t>
         </is>
       </c>
     </row>
@@ -4501,7 +4497,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>[preencher nº]</t>
+          <t>#25236</t>
         </is>
       </c>
     </row>
@@ -4543,11 +4539,17 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>[preencher nº]</t>
+          <t>#25237</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId4"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>